<commit_message>
KPI actualizado 2026-08-25 20:44 UTC
</commit_message>
<xml_diff>
--- a/data/50001586 - ZITRON PERU SAC  CONDESTABLE.xlsx
+++ b/data/50001586 - ZITRON PERU SAC  CONDESTABLE.xlsx
@@ -202,57 +202,57 @@
     <t>Ingenieria Detalle  ot 4387</t>
   </si>
   <si>
+    <t>1217118826919313</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Motor ot 4387</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta Motor  ot 4387 </t>
+  </si>
+  <si>
+    <t>1217303695864968</t>
+  </si>
+  <si>
+    <t>Ingenieria basica nucleo rodete   ot 4387</t>
+  </si>
+  <si>
+    <t>Propuesta Alabes ot 4387,Propuesta rodete ot 4387</t>
+  </si>
+  <si>
+    <t>1217118826927689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ot  4387 -ZVN 1-16-330/4 + TOB + REJ + JF,Ingenieria Jefe de proyecto:,Plano Preliminar   ot 4387  </t>
+  </si>
+  <si>
+    <t>1217117619809504</t>
+  </si>
+  <si>
+    <t>Reservas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva rodete  ot 4387 ,Reserva Alabes ot 4387 </t>
+  </si>
+  <si>
+    <t>1217118826927714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva Alabes ot 4387 </t>
+  </si>
+  <si>
+    <t>NATALYA ESPINOZA</t>
+  </si>
+  <si>
+    <t>nespinoza@zitron.com</t>
+  </si>
+  <si>
+    <t>Reservas,o 2 4387 -ZVN 1-16-330/4 + TOB + REJ + JF</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
   </si>
   <si>
-    <t>1217118826919313</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Motor ot 4387</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta Motor  ot 4387 </t>
-  </si>
-  <si>
-    <t>1217303695864968</t>
-  </si>
-  <si>
-    <t>Ingenieria basica nucleo rodete   ot 4387</t>
-  </si>
-  <si>
-    <t>Propuesta Alabes ot 4387,Propuesta rodete ot 4387</t>
-  </si>
-  <si>
-    <t>1217118826927689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ot  4387 -ZVN 1-16-330/4 + TOB + REJ + JF,Ingenieria Jefe de proyecto:,Plano Preliminar   ot 4387  </t>
-  </si>
-  <si>
-    <t>1217117619809504</t>
-  </si>
-  <si>
-    <t>Reservas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva rodete  ot 4387 ,Reserva Alabes ot 4387 </t>
-  </si>
-  <si>
-    <t>1217118826927714</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva Alabes ot 4387 </t>
-  </si>
-  <si>
-    <t>NATALYA ESPINOZA</t>
-  </si>
-  <si>
-    <t>nespinoza@zitron.com</t>
-  </si>
-  <si>
-    <t>Reservas,o 2 4387 -ZVN 1-16-330/4 + TOB + REJ + JF</t>
-  </si>
-  <si>
     <t>1217119013294914</t>
   </si>
   <si>
@@ -286,40 +286,40 @@
     <t>Generacion oc  ot 4387,Propuesta compras:</t>
   </si>
   <si>
+    <t>1217303610147238</t>
+  </si>
+  <si>
+    <t>Propuesta Alabes ot 4387</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC ALABES  ot 4387</t>
+  </si>
+  <si>
+    <t>1217303610147239</t>
+  </si>
+  <si>
+    <t>Propuesta rodete ot 4387</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,generacion componentes  oc rodetes  ot 4387</t>
+  </si>
+  <si>
+    <t>1217303695864946</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Propuesta Fabricación externa  ot 4387 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check Planos   ot 4387  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generacion Oc ot 4387 </t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1217303610147238</t>
-  </si>
-  <si>
-    <t>Propuesta Alabes ot 4387</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC ALABES  ot 4387</t>
-  </si>
-  <si>
-    <t>1217303610147239</t>
-  </si>
-  <si>
-    <t>Propuesta rodete ot 4387</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,generacion componentes  oc rodetes  ot 4387</t>
-  </si>
-  <si>
-    <t>1217303695864946</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propuesta Fabricación externa  ot 4387 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check Planos   ot 4387  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generacion Oc ot 4387 </t>
-  </si>
-  <si>
-    <t>Baja</t>
   </si>
   <si>
     <t>1217117619809508</t>
@@ -1760,9 +1760,11 @@
       <c r="B8" s="5">
         <v>46237.56788935185</v>
       </c>
-      <c r="C8" s="6"/>
+      <c r="C8" s="5">
+        <v>46259.715407129625</v>
+      </c>
       <c r="D8" s="5">
-        <v>46252.55356030093</v>
+        <v>46259.71541803241</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -1797,24 +1799,28 @@
       <c r="Q8" s="6"/>
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="12" t="s">
-        <v>43</v>
+      <c r="T8" s="6">
+        <v>1</v>
+      </c>
+      <c r="U8" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" s="9">
         <v>46237.56797127315</v>
       </c>
-      <c r="C9" s="10"/>
+      <c r="C9" s="9">
+        <v>46259.715388321754</v>
+      </c>
       <c r="D9" s="9">
-        <v>46247.20498152778</v>
+        <v>46259.71540753472</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>26</v>
@@ -1847,7 +1853,7 @@
         <v>38</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Q9" s="9">
         <v>46246</v>
@@ -1859,25 +1865,27 @@
         <v>33</v>
       </c>
       <c r="T9" s="10">
-        <v>0</v>
-      </c>
-      <c r="U9" s="12" t="s">
-        <v>43</v>
+        <v>1</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" s="5">
         <v>46244.588363981486</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46259.71539701389</v>
+      </c>
       <c r="D10" s="5">
-        <v>46248.17733828704</v>
+        <v>46259.71541480324</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>26</v>
@@ -1910,7 +1918,7 @@
         <v>38</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q10" s="5">
         <v>46247</v>
@@ -1922,15 +1930,15 @@
         <v>33</v>
       </c>
       <c r="T10" s="6">
-        <v>0</v>
-      </c>
-      <c r="U10" s="12" t="s">
-        <v>43</v>
+        <v>1</v>
+      </c>
+      <c r="U10" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="9">
         <v>46237.567974537036</v>
@@ -1975,7 +1983,7 @@
         <v>38</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Q11" s="9">
         <v>46248</v>
@@ -1995,7 +2003,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" s="5">
         <v>46237.56789387732</v>
@@ -2005,7 +2013,7 @@
         <v>46244.59245125</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>25</v>
@@ -2029,7 +2037,7 @@
         <v>26</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P12" s="6" t="s">
         <v>26</v>
@@ -2042,7 +2050,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="9">
         <v>46237.56797914352</v>
@@ -2052,16 +2060,16 @@
         <v>46247.20497636574</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I13" s="9">
         <v>46245</v>
@@ -2079,13 +2087,13 @@
         <v>26</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O13" s="10" t="s">
         <v>38</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q13" s="9">
         <v>46246</v>
@@ -2100,7 +2108,7 @@
         <v>0</v>
       </c>
       <c r="U13" s="12" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -2121,10 +2129,10 @@
         <v>26</v>
       </c>
       <c r="G14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I14" s="5">
         <v>46245</v>
@@ -2142,7 +2150,7 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>38</v>
@@ -2163,7 +2171,7 @@
         <v>0</v>
       </c>
       <c r="U14" s="12" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
@@ -2173,9 +2181,11 @@
       <c r="B15" s="9">
         <v>46244.57396097222</v>
       </c>
-      <c r="C15" s="10"/>
+      <c r="C15" s="9">
+        <v>46259.82100844907</v>
+      </c>
       <c r="D15" s="9">
-        <v>46247.20497568287</v>
+        <v>46259.82102393519</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>64</v>
@@ -2184,10 +2194,10 @@
         <v>26</v>
       </c>
       <c r="G15" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I15" s="9">
         <v>46245</v>
@@ -2205,7 +2215,7 @@
         <v>26</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="O15" s="10" t="s">
         <v>38</v>
@@ -2223,10 +2233,10 @@
         <v>33</v>
       </c>
       <c r="T15" s="10">
-        <v>0</v>
-      </c>
-      <c r="U15" s="12" t="s">
-        <v>43</v>
+        <v>1</v>
+      </c>
+      <c r="U15" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
@@ -2285,10 +2295,10 @@
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46249.16983096064</v>
+        <v>46259.71540726852</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
@@ -2318,7 +2328,7 @@
         <v>67</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>70</v>
@@ -2335,23 +2345,23 @@
       <c r="T17" s="10">
         <v>0</v>
       </c>
-      <c r="U17" s="11" t="s">
-        <v>71</v>
+      <c r="U17" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" s="5">
         <v>46244.57445940972</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46252.20071665509</v>
+        <v>46259.715414085644</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
@@ -2381,10 +2391,10 @@
         <v>67</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q18" s="5">
         <v>46251</v>
@@ -2398,32 +2408,32 @@
       <c r="T18" s="6">
         <v>0</v>
       </c>
-      <c r="U18" s="11" t="s">
-        <v>71</v>
+      <c r="U18" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B19" s="9">
         <v>46244.574642708336</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46252.20071686343</v>
+        <v>46259.715415162034</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I19" s="9">
         <v>46248</v>
@@ -2444,10 +2454,10 @@
         <v>67</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q19" s="9">
         <v>46251</v>
@@ -2461,13 +2471,13 @@
       <c r="T19" s="10">
         <v>0</v>
       </c>
-      <c r="U19" s="11" t="s">
-        <v>71</v>
+      <c r="U19" s="12" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" s="5">
         <v>46244.57978112268</v>
@@ -2477,16 +2487,16 @@
         <v>46244.62653376158</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I20" s="5">
         <v>46309</v>
@@ -2507,10 +2517,10 @@
         <v>67</v>
       </c>
       <c r="O20" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="P20" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="P20" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="Q20" s="5">
         <v>46310</v>
@@ -2519,13 +2529,13 @@
         <v>46309</v>
       </c>
       <c r="S20" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T20" s="6">
         <v>0</v>
       </c>
       <c r="U20" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
@@ -2629,13 +2639,13 @@
         <v>46251</v>
       </c>
       <c r="S22" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T22" s="6">
         <v>0</v>
       </c>
       <c r="U22" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
@@ -2680,7 +2690,7 @@
         <v>87</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>93</v>
@@ -2851,13 +2861,13 @@
         <v>46252</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T26" s="6">
         <v>0</v>
       </c>
       <c r="U26" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -2902,7 +2912,7 @@
         <v>100</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P27" s="10" t="s">
         <v>104</v>
@@ -3026,7 +3036,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3071,7 +3081,7 @@
         <v>109</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>114</v>
@@ -3189,13 +3199,13 @@
         <v>46311</v>
       </c>
       <c r="S32" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3210,7 +3220,7 @@
         <v>46244.62690074074</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
@@ -3240,7 +3250,7 @@
         <v>119</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>124</v>
@@ -3293,7 +3303,7 @@
         <v>119</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P34" s="6" t="s">
         <v>127</v>
@@ -3460,7 +3470,7 @@
         <v>46251</v>
       </c>
       <c r="S37" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T37" s="10">
         <v>1</v>
@@ -3580,7 +3590,7 @@
         <v>46288</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -3656,7 +3666,7 @@
         <v>46252.98552188657</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
@@ -3698,13 +3708,13 @@
         <v>46308</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T41" s="10">
         <v>0</v>
       </c>
       <c r="U41" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -3746,13 +3756,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>146</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
@@ -3814,13 +3824,13 @@
         <v>46379</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T43" s="10">
         <v>0</v>
       </c>
       <c r="U43" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -4030,13 +4040,13 @@
         <v>46247</v>
       </c>
       <c r="S47" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T47" s="10">
         <v>0</v>
       </c>
       <c r="U47" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
@@ -4134,7 +4144,7 @@
         <v>165</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P49" s="10" t="s">
         <v>165</v>
@@ -4205,7 +4215,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4368,13 +4378,13 @@
         <v>46247</v>
       </c>
       <c r="S53" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T53" s="10">
         <v>0</v>
       </c>
       <c r="U53" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4439,7 +4449,7 @@
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="9">
-        <v>46248.174778472225</v>
+        <v>46259.82101358796</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>65</v>
@@ -4537,13 +4547,13 @@
         <v>46352</v>
       </c>
       <c r="S56" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T56" s="6">
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4611,10 +4621,10 @@
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I58" s="5">
         <v>46248</v>
@@ -4647,13 +4657,13 @@
         <v>46248</v>
       </c>
       <c r="S58" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T58" s="6">
         <v>0</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -4674,10 +4684,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I59" s="9">
         <v>46248</v>
@@ -4727,10 +4737,10 @@
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I60" s="5">
         <v>46342</v>
@@ -4780,10 +4790,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H61" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H61" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I61" s="9">
         <v>46251</v>
@@ -4816,13 +4826,13 @@
         <v>46251</v>
       </c>
       <c r="S61" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T61" s="10">
         <v>0</v>
       </c>
       <c r="U61" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -4843,10 +4853,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I62" s="5">
         <v>46251</v>
@@ -4896,10 +4906,10 @@
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H63" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H63" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I63" s="9">
         <v>46339</v>
@@ -4949,10 +4959,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I64" s="5">
         <v>46248</v>
@@ -4985,13 +4995,13 @@
         <v>46248</v>
       </c>
       <c r="S64" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T64" s="6">
         <v>0</v>
       </c>
       <c r="U64" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5012,10 +5022,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H65" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I65" s="9">
         <v>46248</v>
@@ -5065,10 +5075,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I66" s="5">
         <v>46372</v>
@@ -5118,10 +5128,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I67" s="9">
         <v>46374</v>
@@ -5154,13 +5164,13 @@
         <v>46374</v>
       </c>
       <c r="S67" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T67" s="10">
         <v>0</v>
       </c>
       <c r="U67" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5181,10 +5191,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I68" s="5">
         <v>46374</v>
@@ -5234,10 +5244,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I69" s="9">
         <v>46374</v>
@@ -5287,10 +5297,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I70" s="5">
         <v>46377</v>
@@ -5323,13 +5333,13 @@
         <v>46377</v>
       </c>
       <c r="S70" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T70" s="6">
         <v>0</v>
       </c>
       <c r="U70" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5456,10 +5466,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I73" s="9">
         <v>46378</v>
@@ -5492,13 +5502,13 @@
         <v>46378</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T73" s="10">
         <v>0</v>
       </c>
       <c r="U73" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5519,10 +5529,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I74" s="5">
         <v>46378</v>
@@ -5572,10 +5582,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I75" s="9">
         <v>46378</v>
@@ -5625,10 +5635,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I76" s="5">
         <v>46384</v>
@@ -5661,13 +5671,13 @@
         <v>46384</v>
       </c>
       <c r="S76" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T76" s="6">
         <v>0</v>
       </c>
       <c r="U76" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -5688,10 +5698,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I77" s="9">
         <v>46384</v>
@@ -5741,10 +5751,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I78" s="5">
         <v>46384</v>
@@ -5877,13 +5887,13 @@
         <v>46385</v>
       </c>
       <c r="S80" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T80" s="6">
         <v>0</v>
       </c>
       <c r="U80" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6010,10 +6020,10 @@
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H83" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H83" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I83" s="9">
         <v>46386</v>
@@ -6046,13 +6056,13 @@
         <v>46386</v>
       </c>
       <c r="S83" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T83" s="10">
         <v>0</v>
       </c>
       <c r="U83" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
@@ -6073,10 +6083,10 @@
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="H84" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="I84" s="5">
         <v>46386</v>
@@ -6126,10 +6136,10 @@
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H85" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H85" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="I85" s="9">
         <v>46386</v>
@@ -6215,13 +6225,13 @@
         <v>46391</v>
       </c>
       <c r="S86" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T86" s="6">
         <v>0</v>
       </c>
       <c r="U86" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6384,13 +6394,13 @@
         <v>46392</v>
       </c>
       <c r="S89" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T89" s="10">
         <v>0</v>
       </c>
       <c r="U89" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -6600,13 +6610,13 @@
         <v>46393</v>
       </c>
       <c r="S93" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T93" s="10">
         <v>0</v>
       </c>
       <c r="U93" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
@@ -6663,13 +6673,13 @@
         <v>46393</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="11" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>